<commit_message>
Insider redesign: corrected role rules, gatekeeper exclusion, ring signature
Implements Insider Experiment Design!B3-B7: one active gatekeeper set per
run, never C/F/I; B/E/H may coincide with C/F/I (lottery hold, then
local delivery); unconditional 3-way fan-out with 2-of-3 quorum (the
first run's fan-out-to-2 path is removed); and an AOS ring signature over
the 17-node C-candidate pool on libsodium's Ed25519 operations. The
ring-signed GK leg is 801 B raw and padded in its own size class. Moves
the first run's summaries to results/first_run/ as the fixed baseline.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01TXJ7s8Q6PbdYqCeuNUfpZe
</commit_message>
<xml_diff>
--- a/InsiderCompromiseExperiment/Birthmark_Insider_Compromise_Catalog.xlsx
+++ b/InsiderCompromiseExperiment/Birthmark_Insider_Compromise_Catalog.xlsx
@@ -11,7 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Leg Catalog" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Simulation Parameters" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Size Verification" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insider Experiment Design" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insider Results" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Insider Experiment Design" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -170,7 +171,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
@@ -243,6 +244,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -609,7 +614,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A22"/>
+  <dimension ref="A1:A23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -635,7 +640,7 @@
     <row r="4" ht="16" customHeight="1">
       <c r="A4" s="10" t="inlineStr">
         <is>
-          <t>This catalog shares its system-level tabs (Leg Catalog, Simulation Parameters, Size Verification) with the separate GPA traffic-analysis experiment (GPAExperiment/level3/) -- the protocol being described hasn't changed, only the adversary being tested against it. This document's own, distinct content is the Insider Experiment Design tab: a compromised network element holding real keys and exact self-knowledge of its own timing, rather than an outside observer with no keys inferring timing from the network.</t>
+          <t>This catalog shares its system-level tabs (Leg Catalog, Simulation Parameters, Size Verification) with the separate GPA traffic-analysis experiment (GPAExperiment/level3/) -- the protocol being described hasn't changed, only the adversary being tested against it. This document's own content is split across two tabs: Insider Results records what the first run found (a real, confident break for a compromised F or I); Insider Experiment Design specifies the corrected next run, redesigned around that finding.</t>
         </is>
       </c>
     </row>
@@ -673,73 +678,80 @@
     <row r="10" ht="16" customHeight="1">
       <c r="A10" s="10" t="inlineStr">
         <is>
-          <t>Insider Experiment Design -- this catalog's own content: the compromised-element scenarios, the fixed screening point, the two-tier methodology, and what's reused from the GPA experiment's infrastructure.</t>
+          <t>Insider Results -- what the first run found: a compromised F or I confidently beats 1/L, C stays safe, and why. Kept as the baseline the redesign is measured against, including a role-rule error found and corrected.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="10" t="n"/>
+      <c r="A11" s="10" t="inlineStr">
+        <is>
+          <t>Insider Experiment Design -- the corrected spec for the next run: role rules, the gatekeeper exclusion, the reverted gatekeeper fan-out, the ring-signature mitigation, and the device-count sweep, each with a stated rationale and, where relevant, a flagged assumption rather than a silent default.</t>
+        </is>
+      </c>
     </row>
     <row r="12" ht="16" customHeight="1">
-      <c r="A12" s="11" t="inlineStr">
+      <c r="A12" s="10" t="n"/>
+    </row>
+    <row r="13" ht="16" customHeight="1">
+      <c r="A13" s="11" t="inlineStr">
         <is>
           <t>How this relates to the GPA experiment's three levels of test</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="16" customHeight="1">
-      <c r="A13" s="10" t="inlineStr">
+    <row r="14" ht="16" customHeight="1">
+      <c r="A14" s="10" t="inlineStr">
         <is>
           <t>The GPA experiment (GPAExperiment/level3/) tests an outside observer with no key access across three levels: cryptographic distinguishability, protocol/flow distinguishability, and global statistical correlation. This experiment isn't a fourth level in that same progression -- it's a different axis entirely, an adversary with real key access instead of none. Deliberately not called "Level 4" for that reason.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="16" customHeight="1">
-      <c r="A14" s="10" t="n"/>
-    </row>
     <row r="15" ht="16" customHeight="1">
-      <c r="A15" s="11" t="inlineStr">
+      <c r="A15" s="10" t="n"/>
+    </row>
+    <row r="16" ht="16" customHeight="1">
+      <c r="A16" s="11" t="inlineStr">
         <is>
           <t>A/B/C/D/E/F/G/H/I are position labels, not server identities</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="16" customHeight="1">
-      <c r="A16" s="10" t="inlineStr">
+    <row r="17" ht="16" customHeight="1">
+      <c r="A17" s="10" t="inlineStr">
         <is>
           <t>Every letter in Figure 1 (Addressed, Random, and Designated for each channel) names a role-slot for one transaction, filled by whichever node the routing assignment or operator-pool rotation selects that time -- never a fixed, dedicated server. That's why the content-channel Leg IDs are ContA and ContB rather than named after a specific designated-endpoint letter: the leg ID names the channel, independent of which node ever plays a role in delivering it. The Origin/Destination columns still show concrete letters for one example transaction, for legibility -- don't read them as fixed points. The same logic applies to gatekeeper slot assignments (GK-1/2/3) and their transit keys.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="16" customHeight="1">
-      <c r="A17" s="10" t="n"/>
-    </row>
     <row r="18" ht="16" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+      <c r="A18" s="10" t="n"/>
+    </row>
+    <row r="19" ht="16" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>Transit key vs. payload key</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="16" customHeight="1">
-      <c r="A19" s="10" t="inlineStr">
+    <row r="20" ht="16" customHeight="1">
+      <c r="A20" s="10" t="inlineStr">
         <is>
           <t>Every relay hop carries two things: the payload (opaque to every relay node, readable only at the designated endpoint) and, for the first two hops only, a routing code telling the next hop where final delivery should go. Both travel together, encrypted under that hop's own transit key. The device encrypts the routing code together with the still-further-encrypted payload for the first hop; that hop decrypts only the outer layer, reads the routing code, and re-encrypts both for the second hop, whose selection is random and independent of the routing code. The second hop reads the routing code (this is where it's actually used, to know where the Designated hop should deliver) and forwards just the payload, routing code now consumed, to the Designated endpoint. The payload's own encryption is never touched by either intermediate hop.</t>
         </is>
       </c>
     </row>
-    <row r="20" ht="16" customHeight="1">
-      <c r="A20" s="10" t="n"/>
-    </row>
     <row r="21" ht="16" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
+      <c r="A21" s="10" t="n"/>
+    </row>
+    <row r="22" ht="16" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
         <is>
           <t>Design principle</t>
         </is>
       </c>
     </row>
-    <row r="22" ht="16" customHeight="1">
-      <c r="A22" s="10" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="10" t="inlineStr">
         <is>
           <t>Prefer named, established methods over bespoke ones wherever a choice exists -- a named method is independently checkable by a reviewer rather than needing to be justified from scratch. Reflected throughout: Substrate's own transport encryption over inventing one, RFC 7685's established padding range, the Hungarian algorithm for matching, Tor/Shadow's measurement-calibrated traffic model.</t>
         </is>
@@ -2685,6 +2697,144 @@
   <dimension ref="A1:C7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="62" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="17" t="inlineStr">
+        <is>
+          <t>Finding</t>
+        </is>
+      </c>
+      <c r="B1" s="17" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="C1" s="17" t="inlineStr">
+        <is>
+          <t>Read</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="110" customHeight="1">
+      <c r="A2" s="24" t="inlineStr">
+        <is>
+          <t>Headline (first run, superseded design)</t>
+        </is>
+      </c>
+      <c r="B2" s="7" t="inlineStr">
+        <is>
+          <t>A compromised F or I, combined with the network view, links its content to the credential transaction that produced it confidently and far above 1/L: 85% at L=4 down to 33% at L=40 (3.4x-13x baseline), with every top-decile prediction correct at L=4 and L=8. C compromised stays under 1/L at every setting. This run used the design now being replaced (see Insider Experiment Design); results are kept here as the baseline the redesign is measured against.</t>
+        </is>
+      </c>
+      <c r="C2" s="31" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="110" customHeight="1">
+      <c r="A3" s="24" t="inlineStr">
+        <is>
+          <t>Root cause: two compounding pathways</t>
+        </is>
+      </c>
+      <c r="B3" s="7" t="inlineStr">
+        <is>
+          <t>(1) Identity disclosure: F/I must verify C's signature to confirm quorum, which necessarily reveals which node C was. Identity alone (no timing) already scores 50% at L=4 vs. a 25% baseline. (2) Gatekeeper overlap: when the compromised node was itself one of the transaction's gatekeepers (14-17% of items), it received C's fan-out directly, adding 6-17 points on top. Identity disclosure was the dominant effect; gatekeeper overlap was the smaller, additional one.</t>
+        </is>
+      </c>
+      <c r="C3" s="31" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="110" customHeight="1">
+      <c r="A4" s="24" t="inlineStr">
+        <is>
+          <t>C stays safe, and why</t>
+        </is>
+      </c>
+      <c r="B4" s="7" t="inlineStr">
+        <is>
+          <t>C compromised sits at 1.8-2.1x the GPA sequencing attack, under 1/L at every setting, uncalibrated. Nothing on the content side discloses an identity to C the way C's own signature discloses an identity to F/I. This is a structural asymmetry in the protocol, not a modeling artifact.</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="110" customHeight="1">
+      <c r="A5" s="24" t="inlineStr">
+        <is>
+          <t>Relationship to Property F</t>
+        </is>
+      </c>
+      <c r="B5" s="7" t="inlineStr">
+        <is>
+          <t>Property F's literal claim (the credential channel never reaches a content-channel server) remains true. This result shows that claim doesn't deliver the broader device-content non-correlation guarantee, because C's identity leaks through a structurally necessary path (signature verification) a symbolic, timing-blind model was never positioned to catch. This is the first test of A_PRIV's full capability (key access plus network monitoring, granted together per Section 4.1) rather than each half separately.</t>
+        </is>
+      </c>
+      <c r="C5" s="31" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="110" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
+        <is>
+          <t>Not user identity disclosure</t>
+        </is>
+      </c>
+      <c r="B6" s="7" t="inlineStr">
+        <is>
+          <t>A correct pairing reveals which validator authenticated the device, not which device. The token stays encrypted (Section 3.2); only the validator can open it. Recovering an actual device identity still requires compromising (C and V, for the token) or (a device's own first-hop-and-second-hop pair, for its IP), neither of which this result grants on its own.</t>
+        </is>
+      </c>
+      <c r="C6" s="30" t="inlineStr">
+        <is>
+          <t>PASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="110" customHeight="1">
+      <c r="A7" s="24" t="inlineStr">
+        <is>
+          <t>Role-rule error found in this run</t>
+        </is>
+      </c>
+      <c r="B7" s="7" t="inlineStr">
+        <is>
+          <t>This run excluded B from being C, E from being F, and H from being I. The protocol owner confirmed no such exclusion exists or is enforceable: a node acting as B cannot confirm it is later acting as C, since B never decrypts anything and C's later decryption gives it no way to cross-reference. The corrected role rule (Insider Experiment Design) removes this exclusion.</t>
+        </is>
+      </c>
+      <c r="C7" s="31" t="inlineStr">
+        <is>
+          <t>WATCH</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:C9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
     <col width="62" customWidth="1" min="2" max="2"/>
     <col width="42" customWidth="1" min="3" max="3"/>
@@ -2707,100 +2857,131 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="130" customHeight="1">
-      <c r="A2" s="24" t="inlineStr">
+    <row r="2" ht="150" customHeight="1">
+      <c r="A2" s="25" t="inlineStr">
         <is>
           <t>Adversary model</t>
         </is>
       </c>
-      <c r="B2" s="7" t="inlineStr">
-        <is>
-          <t>A single compromised network element (F, I, or C) holding its own real cryptographic keys and exact, zero-noise self-knowledge of its own event timing (when it received content, when it detected quorum, when it posted) -- not inferred from network observation, known directly. Compromise is single-component only, matching A_PRIV's existing threshold; the compromised party gains no other party's keys.</t>
-        </is>
-      </c>
-      <c r="C2" s="7" t="inlineStr">
-        <is>
-          <t>Tests a gap neither existing effort covers: ProVerif proves this adversary can't cryptographically decrypt or correlate device-to-content; the GPA experiment (GPAExperiment/level3/) tested statistical timing correlation but only for an adversary with zero key access. Nobody has tested whether the same compromised key-holder gains anything extra by adding statistical timing analysis on top of what its compromise already grants.</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="130" customHeight="1">
-      <c r="A3" s="24" t="inlineStr">
-        <is>
-          <t>Compromise scenarios, in priority order</t>
-        </is>
-      </c>
-      <c r="B3" s="7" t="inlineStr">
-        <is>
-          <t>1. F compromised. 2. I compromised. 3. C compromised. Relay-node compromise (A, B, D, etc.) deferred -- the routing_code disclosure from a compromised relay node was already reasoned through and accepted as a known, bounded disclosure; worth measuring eventually, not the place to start.</t>
-        </is>
-      </c>
-      <c r="C3" s="7" t="inlineStr">
-        <is>
-          <t>F/I are implicated in the one residual signal the GPA experiment already found (the sequencing attack) -- a compromised F or I has strictly better information than the outside observer had for that same attack, making this the most likely place to find a real signal if one exists. C is the second-most-plausible candidate for the same reason, applied to the credential side.</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="130" customHeight="1">
-      <c r="A4" s="24" t="inlineStr">
-        <is>
-          <t>Fixed point for the screening tier</t>
-        </is>
-      </c>
-      <c r="B4" s="7" t="inlineStr">
-        <is>
-          <t>L = 4 (the smallest anonymity set in the original sweep). All other adopted settings held at their validated values: 25 background clients/node, relay-node shared clock, device per-channel phase, F/I hold before posting.</t>
-        </is>
-      </c>
-      <c r="C4" s="7" t="inlineStr">
-        <is>
-          <t>L=4 was consistently the most attacker-favorable point for the outside GPA across every original result, so it's the worst case for the defender to screen at. Other parameters are fixed at already-validated settings, not arbitrary convenient ones -- background volume was sensitivity-tested and shown not to matter; the three clock/hold mechanisms are the actual adopted design being tested for robustness, not nuisance parameters.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="130" customHeight="1">
-      <c r="A5" s="24" t="inlineStr">
-        <is>
-          <t>Two-tier methodology</t>
-        </is>
-      </c>
-      <c r="B5" s="7" t="inlineStr">
-        <is>
-          <t>Tier 1 (screen): run each compromise scenario (F, I, C) at the single fixed L=4 point. Tier 2 (follow-up): only for a scenario showing a signal materially stronger than what's already known, run a small additional sweep across a few more L values -- not the full 15-setting grid -- to see whether that signal grows, shrinks, or holds steady as L increases.</t>
-        </is>
-      </c>
-      <c r="C5" s="7" t="inlineStr">
-        <is>
-          <t>Keeps compute cost down for the common case (most scenarios likely show nothing new) without silently assuming the fixed-L result generalizes for whichever scenario turns out to matter. The insider's advantage over the outside GPA is a different mechanism (exact self-knowledge vs. inferred observation) and isn't assumed to scale with L the same way the original attack did.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="130" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+      <c r="B2" s="12" t="inlineStr">
+        <is>
+          <t>Unchanged from the first run: a single compromised network element (F, I, or C) holding its own real keys and exact self-knowledge of its own event timing. No other party's keys are granted.</t>
+        </is>
+      </c>
+      <c r="C2" s="33" t="n"/>
+    </row>
+    <row r="3" ht="150" customHeight="1">
+      <c r="A3" s="25" t="inlineStr">
+        <is>
+          <t>Role rules, corrected</t>
+        </is>
+      </c>
+      <c r="B3" s="12" t="inlineStr">
+        <is>
+          <t>Only three hard constraints hold: A cannot be B or C; D cannot be E or F; G cannot be H or I. B, E, and H are otherwise free to coincide with C, F, or I respectively -- the first run's exclusion of this overlap was wrong and is removed.</t>
+        </is>
+      </c>
+      <c r="C3" s="12" t="inlineStr">
+        <is>
+          <t>A node acting as B never decrypts anything (it only reads routing_code and relays an opaque payload); it has no way to later confirm it is the same node now acting as C, since C's decryption gives it nothing to cross-reference against. Confirming the overlap would require active logging across roles, a stronger threat than a single compromised component simply knowing what it legitimately sees. Consistent with how ordinary relay-role overlap is already treated as harmless elsewhere in this catalog.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="150" customHeight="1">
+      <c r="A4" s="25" t="inlineStr">
+        <is>
+          <t>Gatekeeper exclusion from C/F/I</t>
+        </is>
+      </c>
+      <c r="B4" s="12" t="inlineStr">
+        <is>
+          <t>Active gatekeepers can never be assigned the role of C, F, or I. The device table's routing distribution is updated to match the current gatekeeper rotation, so the excluded set stays current as gatekeepers rotate. Pool for these three roles drops from 20 to 17. Gatekeepers can still serve as ordinary relay hops (A/B/D/E/G/H) -- that overlap remains harmless for the same reason given above.</t>
+        </is>
+      </c>
+      <c r="C4" s="12" t="inlineStr">
+        <is>
+          <t>Closes the direct fan-out disclosure pathway completely: if F or I can never be a gatekeeper, it can never directly receive C's fan-out message and learn C's identity that way. This is a routing rule, not a cryptographic one, and its correctness is simple arithmetic (20 minus 3 active gatekeepers), unlike the ring-signature mitigation below. Managing the transition as gatekeepers rotate is real engineering, explicitly out of scope for this paper.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="150" customHeight="1">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
+          <t>Gatekeeper fan-out: reverted to original</t>
+        </is>
+      </c>
+      <c r="B5" s="12" t="inlineStr">
+        <is>
+          <t>C fans out to all 3 selected gatekeepers, unconditionally. The "fan out to only 2" variant tested after the first run is dropped.</t>
+        </is>
+      </c>
+      <c r="C5" s="12" t="inlineStr">
+        <is>
+          <t>That variant existed to reduce two problems that no longer exist under the gatekeeper exclusion above: C signing for itself (impossible now, since C is drawn from the 17-node pool that excludes gatekeepers entirely) and F/I overlap with a gatekeeper (already fully closed by the same exclusion, independent of fan-out count). Reverting restores the original design's availability margin (one gatekeeper can be unavailable without losing quorum) at no remaining cost, and keeps the quorum mechanism exactly the 3-gatekeeper, 2-of-3 structure Property I's existing proofs (BM_Quorum_Forgery.pv, BM_Quorum_Collusion.pv) already cover, rather than introducing an unverified 2-of-2 case.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="150" customHeight="1">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Ring-signature mitigation for C's own signature</t>
+        </is>
+      </c>
+      <c r="B6" s="34" t="inlineStr">
+        <is>
+          <t>C signs as a member of the eligible C-candidate pool (the 17-node pool, minus whatever else is excluded for that specific transaction) rather than with a uniquely identifiable key. F/I verify that a legitimate pool member produced the signature without learning which one. The gatekeeper's own countersignature is unchanged; only C's underlying signature is ring-signed.</t>
+        </is>
+      </c>
+      <c r="C6" s="34" t="inlineStr">
+        <is>
+          <t>Targets the dominant leak the first run found: verifying C's specific signature is what necessarily reveals C's identity to F/I, independent of gatekeeper overlap. Identity-only disclosure scored 50% at L=4 with no timing involved, well above the 25% baseline -- this was the larger of the two pathways, not the smaller one the gatekeeper exclusion addresses. This is a real cryptographic primitive requiring new key material and implementation, not a routing rule, so its effect is measured rather than assumed: expect the full-variant result to collapse toward the timing-only floor (already confirmed under 1/L in every scenario) if it works as intended.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="200" customHeight="1">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
+          <t>Scale: device counts and the L relationship</t>
+        </is>
+      </c>
+      <c r="B7" s="34" t="inlineStr">
+        <is>
+          <t>Three device counts: 80, 240, 400. Interval held fixed at the original 20 minutes, so L scales naturally with device count (80-&gt;L=8, 240-&gt;L=24, 400-&gt;L=40) rather than being held constant across the three.</t>
+        </is>
+      </c>
+      <c r="C7" s="34" t="inlineStr">
+        <is>
+          <t>Device count and L measure different things -- device count is the size of the identity-disclosure candidate pool (devices per validator), L is temporal overlap -- and the first run's dominant effect was identity disclosure, which L alone doesn't capture. Holding interval fixed lets one sweep carry information about both axes rather than requiring a full cross. FLAGGED ASSUMPTION, not confirmed: if device count and L need to be varied independently instead, this sweep design needs to change to a real cross. These specific L values (8, 24, 40) match points already measured in both the GPA experiment's Tier 2 sweep and the first insider run's own Tier 2 sweep, so this run's results compare directly against both existing datasets at those points without interpolation. The device-count values themselves reflect a floor a real deployment could plausibly maintain via synthetic traffic even with minimal genuine usage, consistent with the GPA experiment's own dummy-traffic-floor methodology.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="150" customHeight="1">
+      <c r="A8" s="25" t="inlineStr">
         <is>
           <t>Success criterion</t>
         </is>
       </c>
-      <c r="B6" s="7" t="inlineStr">
-        <is>
-          <t>Same as the GPA experiment: accuracy vs. the 1/L chance baseline, plus calibration (accuracy among high-confidence predictions specifically).</t>
-        </is>
-      </c>
-      <c r="C6" s="7" t="inlineStr">
-        <is>
-          <t>Reused rather than redesigned -- the question ("does this adversary gain an actionable pairing capability") is the same shape regardless of what information the adversary starts with.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="130" customHeight="1">
-      <c r="A7" s="24" t="inlineStr">
-        <is>
-          <t>Reused infrastructure</t>
-        </is>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
-        <is>
-          <t>Same simulator, same lottery/clock mechanics, same padding rules as the GPA experiment. The only change is the observer's vantage point: exact self-knowledge of the compromised party's own events, replacing inferred network observation for those specific events. No other party's keys are granted; everything the existing ProVerif proofs already establish about what a single compromised component cannot decrypt still holds.</t>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Unchanged: accuracy against 1/L and against random assignment over the same feasible pairs, the top-vs-runner-up score gap, and accuracy in the top 10% of gaps.</t>
+        </is>
+      </c>
+      <c r="C8" s="33" t="n"/>
+    </row>
+    <row r="9" ht="150" customHeight="1">
+      <c r="A9" s="26" t="inlineStr">
+        <is>
+          <t>Expected outcome, stated in advance</t>
+        </is>
+      </c>
+      <c r="B9" s="34" t="inlineStr">
+        <is>
+          <t>The gatekeeper exclusion should remove the gatekeeper-overlap contribution specifically (roughly the 6-17 points it added in the first run). The ring signature should remove the identity-disclosure contribution (the 50% identity-only floor at L=4). Together, if both work as intended, the full variant should collapse toward the timing-only result, which already stayed under 1/L in every scenario tested.</t>
+        </is>
+      </c>
+      <c r="C9" s="34" t="inlineStr">
+        <is>
+          <t>Stated before running, not after, so a result that doesn't match this prediction is itself flagged as a finding rather than quietly reinterpreted. This project has been wrong about a "should work" prediction before (the CV-1/2 hold, GPA experiment) -- the fix worked eventually, but not the way first assumed.</t>
         </is>
       </c>
     </row>

</xml_diff>